<commit_message>
Tracker: add SAP Hong Kong as watch employer (no HK FG tech role open 2026-10-27)
</commit_message>
<xml_diff>
--- a/documents/HK_Job_Search_Tracker_2026-10-13.xlsx
+++ b/documents/HK_Job_Search_Tracker_2026-10-13.xlsx
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -4013,7 +4014,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>備註：更新於 2026-10-27。CBI Application Developer 亦被 Jobsdb 封鎖，但用戶已決定不投（公司規模小），未列入。</t>
@@ -4041,7 +4041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q113"/>
+  <dimension ref="A1:Q114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12338,6 +12338,82 @@
         <v>46308</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="24" t="inlineStr">
+        <is>
+          <t>T105</t>
+        </is>
+      </c>
+      <c r="B114" s="24" t="inlineStr">
+        <is>
+          <t>SAP 香港</t>
+        </is>
+      </c>
+      <c r="C114" s="24" t="inlineStr">
+        <is>
+          <t>企業軟件/ERP/AI</t>
+        </is>
+      </c>
+      <c r="D114" s="24" t="inlineStr">
+        <is>
+          <t>（暫無香港FG科技崗）</t>
+        </is>
+      </c>
+      <c r="E114" s="24" t="inlineStr">
+        <is>
+          <t>AI/Agent/软件</t>
+        </is>
+      </c>
+      <c r="F114" s="24" t="inlineStr">
+        <is>
+          <t>P3 觀察</t>
+        </is>
+      </c>
+      <c r="G114" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-27查SAP新舊招聘站：香港只有Senior Account Executive（資深銷售）。</t>
+        </is>
+      </c>
+      <c r="H114" s="48" t="n"/>
+      <c r="I114" s="24" t="inlineStr">
+        <is>
+          <t>無香港FG職位，無截止。</t>
+        </is>
+      </c>
+      <c r="J114" s="24" t="inlineStr">
+        <is>
+          <t>亞太畢業生崗在上海/大連（STAR 2028屆）及新加坡實習，不符香港限制。</t>
+        </is>
+      </c>
+      <c r="K114" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L114" s="24" t="inlineStr">
+        <is>
+          <t>出現香港Graduate/FG IT、AI或Data崗再投。</t>
+        </is>
+      </c>
+      <c r="M114" s="26" t="inlineStr">
+        <is>
+          <t>https://careers.sap.com/search/?q=&amp;locationsearch=Hong+Kong</t>
+        </is>
+      </c>
+      <c r="N114" s="24" t="n"/>
+      <c r="O114" s="24" t="inlineStr">
+        <is>
+          <t>用戶2026-10-27要求加入。</t>
+        </is>
+      </c>
+      <c r="P114" s="24">
+        <f>IF(H114="","",H114-'申请追踪'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="Q114" s="48" t="n">
+        <v>46322</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="G10:G57">
     <cfRule type="containsText" priority="1" operator="containsText" dxfId="2" text="已填满"/>

</xml_diff>

<commit_message>
Tracker: add Avenir Group / DeepTrading (2026-10-27 check)
</commit_message>
<xml_diff>
--- a/documents/HK_Job_Search_Tracker_2026-10-13.xlsx
+++ b/documents/HK_Job_Search_Tracker_2026-10-13.xlsx
@@ -4041,7 +4041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q114"/>
+  <dimension ref="A1:Q115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12414,6 +12414,82 @@
         <v>46322</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="24" t="inlineStr">
+        <is>
+          <t>T106</t>
+        </is>
+      </c>
+      <c r="B115" s="24" t="inlineStr">
+        <is>
+          <t>Avenir Group（李林家族辦公室）/ DeepTrading</t>
+        </is>
+      </c>
+      <c r="C115" s="24" t="inlineStr">
+        <is>
+          <t>加密資產投資/高頻交易</t>
+        </is>
+      </c>
+      <c r="D115" s="24" t="inlineStr">
+        <is>
+          <t>DeepTrading Junior C++ Quantitative Systems Engineer（0–3年）</t>
+        </is>
+      </c>
+      <c r="E115" s="24" t="inlineStr">
+        <is>
+          <t>AI/Agent/软件</t>
+        </is>
+      </c>
+      <c r="F115" s="24" t="inlineStr">
+        <is>
+          <t>P2 技能不符</t>
+        </is>
+      </c>
+      <c r="G115" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-27：Avenir 官網無招聘頁，只在LinkedIn招聘；香港現有IR Manager、Senior Treasury BP、Senior Finance Manager、Options Trader，無FG科技崗。子公司DeepTrading長期招Junior C++量化系統工程師（0–3年，全職），辦公室北京+香港，未寫明工作地。</t>
+        </is>
+      </c>
+      <c r="H115" s="48" t="n"/>
+      <c r="I115" s="24" t="inlineStr">
+        <is>
+          <t>長期開放，無截止。</t>
+        </is>
+      </c>
+      <c r="J115" s="24" t="inlineStr">
+        <is>
+          <t>要求精通C++及大型代碼庫，非明確FG字樣；用戶主力為Python/ML，C++不能推定滿足。</t>
+        </is>
+      </c>
+      <c r="K115" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L115" s="24" t="inlineStr">
+        <is>
+          <t>如用戶C++扎實可考慮；電郵AvenirDeepTradingHR@avenirx.com並註明香港。</t>
+        </is>
+      </c>
+      <c r="M115" s="26" t="inlineStr">
+        <is>
+          <t>https://www.avenirdeeptrading.com/en/</t>
+        </is>
+      </c>
+      <c r="N115" s="24" t="n"/>
+      <c r="O115" s="24" t="inlineStr">
+        <is>
+          <t>用戶2026-10-27要求查看。</t>
+        </is>
+      </c>
+      <c r="P115" s="24">
+        <f>IF(H115="","",H115-'申请追踪'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="Q115" s="48" t="n">
+        <v>46322</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="G10:G57">
     <cfRule type="containsText" priority="1" operator="containsText" dxfId="2" text="已填满"/>

</xml_diff>